<commit_message>
chore: add Test-and-Report results
</commit_message>
<xml_diff>
--- a/code/scripts/results/known_growth_phenotypes_w_pred.xlsx
+++ b/code/scripts/results/known_growth_phenotypes_w_pred.xlsx
@@ -487,107 +487,107 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>L1</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Nitrate</t>
+          <t>Kratzl Base Medium</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Acetate</t>
+          <t>Ammonium, Succinate</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>(Kratzl, 2026)</t>
         </is>
       </c>
       <c r="G2" t="n">
-        <v>0.37</v>
+        <v>0</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>True Positive</t>
+          <t>True Negative</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>L1</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Nitrate</t>
+          <t>Kratzl Base Medium</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Alanine</t>
+          <t>Nitrate, Succinate</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>(Kratzl, 2026)</t>
         </is>
       </c>
       <c r="G3" t="n">
-        <v>0.585</v>
+        <v>0</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>True Positive</t>
+          <t>True Negative</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>L1</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Nitrate</t>
+          <t>Kratzl Base Medium</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>DHPS (dihydroxypropanesulfonate)</t>
+          <t>Urea, Succinate</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>(Kratzl, 2026)</t>
         </is>
       </c>
       <c r="G4" t="n">
-        <v>0.583</v>
+        <v>0</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>True Positive</t>
+          <t>True Negative</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>L1</t>
+          <t>Kratzl Base Medium (with N-solution)</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Nitrate</t>
+          <t>NH3, Nitrate</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Glucose</t>
+          <t>Alanine</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -595,8 +595,13 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>(Kratzl, 2026)</t>
+        </is>
+      </c>
       <c r="G5" t="n">
-        <v>0.647</v>
+        <v>0.585</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
@@ -607,17 +612,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>L1</t>
+          <t>Kratzl Base Medium (with N-solution)</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Nitrate</t>
+          <t>NH3, Nitrate</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Glutamate</t>
+          <t>Alanine, Pyruvate</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -625,8 +630,13 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>(Kratzl, 2026)</t>
+        </is>
+      </c>
       <c r="G6" t="n">
-        <v>0.71</v>
+        <v>0.766</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
@@ -637,17 +647,17 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>L1</t>
+          <t>Kratzl Base Medium (with N-solution)</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Nitrate</t>
+          <t>NH3, Nitrate</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Glycerol-3-phosphate</t>
+          <t>Arginine</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -655,8 +665,13 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>(Kratzl, 2026)</t>
+        </is>
+      </c>
       <c r="G7" t="n">
-        <v>0.804</v>
+        <v>0.613</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
@@ -667,17 +682,17 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>L1</t>
+          <t>Kratzl Base Medium (with N-solution)</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Nitrate</t>
+          <t>NH3, Nitrate</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Proline</t>
+          <t>Arginine, Pyruvate</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -685,8 +700,13 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>(Kratzl, 2026)</t>
+        </is>
+      </c>
       <c r="G8" t="n">
-        <v>0.6870000000000001</v>
+        <v>0.78</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
@@ -697,67 +717,78 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>L1</t>
+          <t>Kratzl Base Medium (with N-solution)</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Nitrate</t>
+          <t>NH3, Nitrate</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Tyrosine</t>
+          <t>Cystine</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>(Kratzl, 2026)</t>
         </is>
       </c>
       <c r="G9" t="n">
-        <v>0.327</v>
+        <v>0</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>True Positive</t>
+          <t>True Negative</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>L1</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Nitrate</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Valine</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G10" t="n">
-        <v>0.492</v>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>True Positive</t>
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Kratzl Base Medium (with N-solution)</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>NH3, Nitrate</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Cystine, Pyruvate</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>(Kratzl, 2026)</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr"/>
+      <c r="G10" s="2" t="n">
+        <v>0.5649999999999999</v>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>False Positive</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Marine Broth</t>
+          <t>Kratzl Base Medium (with N-solution)</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -767,7 +798,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Alanine</t>
+          <t>Glutamine</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -781,7 +812,7 @@
         </is>
       </c>
       <c r="G11" t="n">
-        <v>0.585</v>
+        <v>0.719</v>
       </c>
       <c r="H11" t="inlineStr">
         <is>
@@ -792,7 +823,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Marine Broth</t>
+          <t>Kratzl Base Medium (with N-solution)</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -802,7 +833,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Alanine, Pyruvate</t>
+          <t>Glutamine, Pyruvate</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -816,7 +847,7 @@
         </is>
       </c>
       <c r="G12" t="n">
-        <v>0.766</v>
+        <v>0.889</v>
       </c>
       <c r="H12" t="inlineStr">
         <is>
@@ -827,7 +858,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Marine Broth</t>
+          <t>Kratzl Base Medium (with N-solution)</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -837,7 +868,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Arginine</t>
+          <t>Lysine</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -851,7 +882,7 @@
         </is>
       </c>
       <c r="G13" t="n">
-        <v>0.613</v>
+        <v>0.504</v>
       </c>
       <c r="H13" t="inlineStr">
         <is>
@@ -862,7 +893,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Marine Broth</t>
+          <t>Kratzl Base Medium (with N-solution)</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -872,7 +903,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Arginine, Pyruvate</t>
+          <t>Lysine, Pyruvate</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -886,7 +917,7 @@
         </is>
       </c>
       <c r="G14" t="n">
-        <v>0.78</v>
+        <v>0.6919999999999999</v>
       </c>
       <c r="H14" t="inlineStr">
         <is>
@@ -897,7 +928,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Marine Broth</t>
+          <t>Kratzl Base Medium (with N-solution)</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -907,7 +938,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Cystine</t>
+          <t>Methionine</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -930,80 +961,80 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>Marine Broth</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="inlineStr">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Kratzl Base Medium (with N-solution)</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
         <is>
           <t>NH3, Nitrate</t>
         </is>
       </c>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t>Cystine, Pyruvate</t>
-        </is>
-      </c>
-      <c r="D16" s="2" t="inlineStr">
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Methionine, Pyruvate</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>(Kratzl, 2026)</t>
+        </is>
+      </c>
+      <c r="G16" t="n">
+        <v>0.5649999999999999</v>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>True Positive</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Kratzl Base Medium (with N-solution)</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>NH3, Nitrate</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Proline</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="E16" s="2" t="inlineStr">
+      <c r="E17" s="2" t="inlineStr">
         <is>
           <t>(Kratzl, 2026)</t>
         </is>
       </c>
-      <c r="F16" s="2" t="inlineStr"/>
-      <c r="G16" s="2" t="n">
-        <v>0.5649999999999999</v>
-      </c>
-      <c r="H16" s="2" t="inlineStr">
+      <c r="F17" s="2" t="inlineStr"/>
+      <c r="G17" s="2" t="n">
+        <v>0.6870000000000001</v>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
         <is>
           <t>False Positive</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>Marine Broth</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>NH3, Nitrate</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>Glutamine</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>(Kratzl, 2026)</t>
-        </is>
-      </c>
-      <c r="G17" t="n">
-        <v>0.719</v>
-      </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>True Positive</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Marine Broth</t>
+          <t>Kratzl Base Medium (with N-solution)</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1013,7 +1044,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Glutamine, Pyruvate</t>
+          <t>Proline, Pyruvate</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1027,7 +1058,7 @@
         </is>
       </c>
       <c r="G18" t="n">
-        <v>0.889</v>
+        <v>0.852</v>
       </c>
       <c r="H18" t="inlineStr">
         <is>
@@ -1038,17 +1069,17 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Marine Broth</t>
+          <t>L1</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>NH3, Nitrate</t>
+          <t>Nitrate</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Lysine</t>
+          <t>Acetate</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -1056,13 +1087,8 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>(Kratzl, 2026)</t>
-        </is>
-      </c>
       <c r="G19" t="n">
-        <v>0.504</v>
+        <v>0.37</v>
       </c>
       <c r="H19" t="inlineStr">
         <is>
@@ -1073,17 +1099,17 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Marine Broth</t>
+          <t>L1</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>NH3, Nitrate</t>
+          <t>Nitrate</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Lysine, Pyruvate</t>
+          <t>Alanine</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -1091,13 +1117,8 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>(Kratzl, 2026)</t>
-        </is>
-      </c>
       <c r="G20" t="n">
-        <v>0.6919999999999999</v>
+        <v>0.585</v>
       </c>
       <c r="H20" t="inlineStr">
         <is>
@@ -1108,52 +1129,47 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Marine Broth</t>
+          <t>L1</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>NH3, Nitrate</t>
+          <t>Nitrate</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Methionine</t>
+          <t>DHPS (dihydroxypropanesulfonate)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>(Kratzl, 2026)</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G21" t="n">
-        <v>0</v>
+        <v>0.583</v>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>True Negative</t>
+          <t>True Positive</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Marine Broth</t>
+          <t>L1</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>NH3, Nitrate</t>
+          <t>Nitrate</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Methionine, Pyruvate</t>
+          <t>Glucose</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -1161,13 +1177,8 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>(Kratzl, 2026)</t>
-        </is>
-      </c>
       <c r="G22" t="n">
-        <v>0.5649999999999999</v>
+        <v>0.647</v>
       </c>
       <c r="H22" t="inlineStr">
         <is>
@@ -1176,55 +1187,49 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="2" t="inlineStr">
-        <is>
-          <t>Marine Broth</t>
-        </is>
-      </c>
-      <c r="B23" s="2" t="inlineStr">
-        <is>
-          <t>NH3, Nitrate</t>
-        </is>
-      </c>
-      <c r="C23" s="2" t="inlineStr">
-        <is>
-          <t>Proline</t>
-        </is>
-      </c>
-      <c r="D23" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="E23" s="2" t="inlineStr">
-        <is>
-          <t>(Kratzl, 2026)</t>
-        </is>
-      </c>
-      <c r="F23" s="2" t="inlineStr"/>
-      <c r="G23" s="2" t="n">
-        <v>0.6870000000000001</v>
-      </c>
-      <c r="H23" s="2" t="inlineStr">
-        <is>
-          <t>False Positive</t>
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Nitrate</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Glutamate</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G23" t="n">
+        <v>0.71</v>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>True Positive</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Marine Broth</t>
+          <t>L1</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>NH3, Nitrate</t>
+          <t>Nitrate</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Proline, Pyruvate</t>
+          <t>Glycerol-3-phosphate</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -1232,13 +1237,8 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>(Kratzl, 2026)</t>
-        </is>
-      </c>
       <c r="G24" t="n">
-        <v>0.852</v>
+        <v>0.804</v>
       </c>
       <c r="H24" t="inlineStr">
         <is>
@@ -1249,90 +1249,90 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Marine Broth (No Nitrogen)</t>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Nitrate</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Ammonium, Succinate</t>
+          <t>Proline</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>(Kratzl, 2026)</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G25" t="n">
-        <v>0</v>
+        <v>0.6870000000000001</v>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>True Negative</t>
+          <t>True Positive</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Marine Broth (No Nitrogen)</t>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Nitrate</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Nitrate, Succinate</t>
+          <t>Tyrosine</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>(Kratzl, 2026)</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G26" t="n">
-        <v>0</v>
+        <v>0.327</v>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>True Negative</t>
+          <t>True Positive</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Marine Broth (No Nitrogen)</t>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Nitrate</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Urea, Succinate</t>
+          <t>Valine</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>(Kratzl, 2026)</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G27" t="n">
-        <v>0</v>
+        <v>0.492</v>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>True Negative</t>
+          <t>True Positive</t>
         </is>
       </c>
     </row>
@@ -2271,7 +2271,7 @@
     <row r="57">
       <c r="A57" s="3" t="inlineStr">
         <is>
-          <t>Marine Broth (No Nitrogen)</t>
+          <t>Kratzl Base Medium</t>
         </is>
       </c>
       <c r="B57" s="3" t="inlineStr"/>
@@ -2307,7 +2307,7 @@
     <row r="58">
       <c r="A58" s="3" t="inlineStr">
         <is>
-          <t>Marine Broth (No Nitrogen)</t>
+          <t>Kratzl Base Medium</t>
         </is>
       </c>
       <c r="B58" s="3" t="inlineStr"/>
@@ -2343,7 +2343,7 @@
     <row r="59">
       <c r="A59" s="3" t="inlineStr">
         <is>
-          <t>Marine Broth (No Nitrogen)</t>
+          <t>Kratzl Base Medium</t>
         </is>
       </c>
       <c r="B59" s="3" t="inlineStr"/>
@@ -2379,7 +2379,7 @@
     <row r="60">
       <c r="A60" s="3" t="inlineStr">
         <is>
-          <t>Marine Broth (No Nitrogen)</t>
+          <t>Kratzl Base Medium</t>
         </is>
       </c>
       <c r="B60" s="3" t="inlineStr"/>
@@ -2415,7 +2415,7 @@
     <row r="61">
       <c r="A61" s="3" t="inlineStr">
         <is>
-          <t>Marine Broth (No Nitrogen)</t>
+          <t>Kratzl Base Medium</t>
         </is>
       </c>
       <c r="B61" s="3" t="inlineStr"/>
@@ -2451,7 +2451,7 @@
     <row r="62">
       <c r="A62" s="3" t="inlineStr">
         <is>
-          <t>Marine Broth (No Nitrogen)</t>
+          <t>Kratzl Base Medium</t>
         </is>
       </c>
       <c r="B62" s="3" t="inlineStr"/>

</xml_diff>